<commit_message>
style: remove sample participant names from excel template
</commit_message>
<xml_diff>
--- a/template_peserta_nrp_kosong.xlsx
+++ b/template_peserta_nrp_kosong.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="8">
   <si>
     <t>TEMPLATE DAFTAR PESERTA TRAINING</t>
   </si>
@@ -39,42 +39,6 @@
   </si>
   <si>
     <t>Jenis Kelamin</t>
-  </si>
-  <si>
-    <t>Excel Daud</t>
-  </si>
-  <si>
-    <t>E00234</t>
-  </si>
-  <si>
-    <t>Software Engineer</t>
-  </si>
-  <si>
-    <t>Balikpapan</t>
-  </si>
-  <si>
-    <t>08123456789</t>
-  </si>
-  <si>
-    <t>L</t>
-  </si>
-  <si>
-    <t>Jane Doe</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>HR Staff</t>
-  </si>
-  <si>
-    <t>Jakarta</t>
-  </si>
-  <si>
-    <t>08987654321</t>
-  </si>
-  <si>
-    <t>P</t>
   </si>
 </sst>
 </file>
@@ -542,44 +506,20 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="A5" s="4"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="6"/>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>19</v>
-      </c>
+      <c r="A6" s="4"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="6"/>
     </row>
   </sheetData>
   <mergeCells>

</xml_diff>

<commit_message>
feat: implement dual-sheet Excel for participants and organizers
</commit_message>
<xml_diff>
--- a/template_peserta_nrp_kosong.xlsx
+++ b/template_peserta_nrp_kosong.xlsx
@@ -1,99 +1,110 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Excel Daud\Herd\booking\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55CB639D-8DBF-4F7A-9E89-C14366B6C83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="3210" yWindow="4185" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Template Roster" sheetId="1" r:id="rId4"/>
+    <sheet name="Peserta" sheetId="1" r:id="rId1"/>
+    <sheet name="Panitia" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="8">
-  <si>
-    <t>TEMPLATE DAFTAR PESERTA TRAINING</t>
-  </si>
-  <si>
-    <t>Catatan: Jangan mengubah header. Kolom B (NRP) wajib diisi, ketik 'N/A' jika tidak ada. Kolom F hanya 'L' atau 'P'.</t>
-  </si>
-  <si>
-    <t>Nama Lengkap</t>
-  </si>
-  <si>
-    <t>NRP</t>
-  </si>
-  <si>
-    <t>Jabatan</t>
-  </si>
-  <si>
-    <t>Site</t>
-  </si>
-  <si>
-    <t>No HP</t>
-  </si>
-  <si>
-    <t>Jenis Kelamin</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="16">
+  <si>
+    <t>FORMAT DATA PESERTA</t>
+  </si>
+  <si>
+    <t>PENTING: Jangan ubah format baris 1 sampai 4. Data dimulai dari baris ke-5.</t>
+  </si>
+  <si>
+    <t>Nama Lengkap (Wajib)</t>
+  </si>
+  <si>
+    <t>NRP (Wajib, isi N/A jika tidak ada)</t>
+  </si>
+  <si>
+    <t>Jabatan (Wajib)</t>
+  </si>
+  <si>
+    <t>Site (Wajib)</t>
+  </si>
+  <si>
+    <t>No. HP (Wajib, angka)</t>
+  </si>
+  <si>
+    <t>Jenis Kelamin (L/P)</t>
+  </si>
+  <si>
+    <t>Contoh Nama Peserta</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Staff</t>
+  </si>
+  <si>
+    <t>HO</t>
+  </si>
+  <si>
+    <t>081234567890</t>
+  </si>
+  <si>
+    <t>L</t>
+  </si>
+  <si>
+    <t>FORMAT DATA PANITIA</t>
+  </si>
+  <si>
+    <t>Contoh Nama Panitia</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="12"/>
-      <color rgb="FFFFFFFF"/>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="0"/>
-      <i val="1"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="9"/>
-      <color rgb="FF991B1B"/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
-      <sz val="10"/>
-      <color rgb="FF555555"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -102,24 +113,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF1E3A5F"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2563EB"/>
+        <fgColor rgb="FFD9D9D9"/>
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -127,49 +126,30 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="2" numFmtId="0" fillId="3" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="3" numFmtId="0" fillId="4" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="0"/>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="4" numFmtId="0" fillId="0" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -459,75 +439,165 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30" customWidth="true" style="0"/>
-    <col min="2" max="2" width="18" customWidth="true" style="0"/>
-    <col min="3" max="3" width="25" customWidth="true" style="0"/>
-    <col min="4" max="4" width="18" customWidth="true" style="0"/>
-    <col min="5" max="5" width="20" customWidth="true" style="0"/>
-    <col min="6" max="6" width="18" customWidth="true" style="0"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="31.28515625" customWidth="1"/>
+    <col min="3" max="3" width="23.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" customWidth="1"/>
+    <col min="6" max="6" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" customHeight="1" ht="32">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" customHeight="1" ht="24">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" customHeight="1" ht="10"/>
-    <row r="4" spans="1:6" customHeight="1" ht="24">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="4"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="6"/>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="4"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="6"/>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells>
+  <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
   </mergeCells>
-  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="27.85546875" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" customWidth="1"/>
+    <col min="4" max="4" width="23.28515625" customWidth="1"/>
+    <col min="5" max="5" width="27.42578125" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>